<commit_message>
Dimensionality analyses saves correlation matrix with row- and colnames Dimensionality tables for technical reports can handle user-supplied row- and column names and reorder table rows and columns Fixture for dimensionality analyse with data example 2 rerun to create new exported files Adapted tests for TblDim()
</commit_message>
<xml_diff>
--- a/tests/testthat/fixtures/ex2/tables/dimensionality.xlsx
+++ b/tests/testthat/fixtures/ex2/tables/dimensionality.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -25,40 +25,43 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">V2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V4</t>
+    <t xml:space="preserve">units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Npars</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
+    <t xml:space="preserve">loglik</t>
+  </si>
+  <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
+    <t xml:space="preserve">AIC</t>
+  </si>
+  <si>
     <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">uni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">content</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Npars</t>
-  </si>
-  <si>
-    <t xml:space="preserve">loglik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIC</t>
   </si>
   <si>
     <t xml:space="preserve">BIC</t>
@@ -403,7 +406,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>1.51</v>
+        <v>1.597</v>
       </c>
     </row>
   </sheetData>
@@ -422,84 +425,84 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>2.04</v>
+        <v>2.003</v>
       </c>
       <c r="C2" t="n">
-        <v>0.673</v>
+        <v>0.737</v>
       </c>
       <c r="D2" t="n">
-        <v>0.744</v>
+        <v>0.749</v>
       </c>
       <c r="E2" t="n">
-        <v>0.751</v>
+        <v>0.775</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>0.673</v>
+        <v>0.737</v>
       </c>
       <c r="C3" t="n">
-        <v>2.185</v>
+        <v>2.359</v>
       </c>
       <c r="D3" t="n">
-        <v>0.712</v>
+        <v>0.718</v>
       </c>
       <c r="E3" t="n">
-        <v>0.725</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.744</v>
+        <v>0.749</v>
       </c>
       <c r="C4" t="n">
-        <v>0.712</v>
+        <v>0.718</v>
       </c>
       <c r="D4" t="n">
-        <v>2.876</v>
+        <v>2.887</v>
       </c>
       <c r="E4" t="n">
-        <v>0.701</v>
+        <v>0.704</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>0.751</v>
+        <v>0.775</v>
       </c>
       <c r="C5" t="n">
-        <v>0.725</v>
+        <v>0.75</v>
       </c>
       <c r="D5" t="n">
-        <v>0.701</v>
+        <v>0.704</v>
       </c>
       <c r="E5" t="n">
-        <v>2.391</v>
+        <v>2.397</v>
       </c>
     </row>
   </sheetData>
@@ -518,13 +521,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
         <v>9</v>
-      </c>
-      <c r="C1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2">
@@ -532,7 +535,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
         <v>24</v>
@@ -543,44 +546,44 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>-13183</v>
+        <v>-13032</v>
       </c>
       <c r="D3" t="n">
-        <v>-13092</v>
+        <v>-12955</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
       </c>
       <c r="C4" t="n">
-        <v>26414</v>
+        <v>26112</v>
       </c>
       <c r="D4" t="n">
-        <v>26250</v>
+        <v>25976</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>26542</v>
+        <v>26240</v>
       </c>
       <c r="D5" t="n">
-        <v>26425</v>
+        <v>26151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>